<commit_message>
Se tiene un respaldo de los Eventos y Cuentas en un archivo PICKL, hay q revisar los porcentajes de las cuentas, por lo demas funciona
</commit_message>
<xml_diff>
--- a/models/hora_extra_template.xlsx
+++ b/models/hora_extra_template.xlsx
@@ -12,7 +12,7 @@
     <sheet name="result" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">result!$A$1:$M$180</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">result!$A$1:$N$1</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="76">
   <si>
     <t xml:space="preserve">Aplica</t>
   </si>
@@ -249,6 +249,9 @@
   </si>
   <si>
     <t xml:space="preserve">Archivo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tipo</t>
   </si>
 </sst>
 </file>
@@ -429,7 +432,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -499,23 +502,27 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -555,18 +562,10 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -1311,7 +1310,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M811"/>
+  <dimension ref="A1:N811"/>
   <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="17" width="31.57"/>
@@ -1321,198 +1320,202 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="20" width="14.57"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="20" width="13.42"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="21" width="19.71"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="17" width="170.29"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="22" width="170.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="12.29"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="11" style="1" width="10.14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="55.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="22.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="1" width="13.42"/>
   </cols>
   <sheetData>
-    <row r="1" s="22" customFormat="true" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="22" t="s">
+    <row r="1" s="23" customFormat="true" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="23" t="s">
         <v>63</v>
       </c>
-      <c r="B1" s="22" t="s">
+      <c r="B1" s="23" t="s">
         <v>64</v>
       </c>
-      <c r="C1" s="22" t="s">
+      <c r="C1" s="23" t="s">
         <v>65</v>
       </c>
-      <c r="D1" s="23" t="s">
+      <c r="D1" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="24" t="s">
+      <c r="E1" s="25" t="s">
         <v>66</v>
       </c>
-      <c r="F1" s="24" t="s">
+      <c r="F1" s="25" t="s">
         <v>67</v>
       </c>
-      <c r="G1" s="25" t="s">
+      <c r="G1" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="H1" s="22" t="s">
+      <c r="H1" s="23" t="s">
         <v>69</v>
       </c>
-      <c r="I1" s="22" t="s">
+      <c r="I1" s="23" t="s">
         <v>70</v>
       </c>
-      <c r="J1" s="22" t="s">
+      <c r="J1" s="23" t="s">
         <v>71</v>
       </c>
-      <c r="K1" s="22" t="s">
+      <c r="K1" s="23" t="s">
         <v>72</v>
       </c>
-      <c r="L1" s="22" t="s">
+      <c r="L1" s="23" t="s">
         <v>73</v>
       </c>
-      <c r="M1" s="22" t="s">
+      <c r="M1" s="23" t="s">
         <v>74</v>
       </c>
+      <c r="N1" s="23" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H2" s="26"/>
+      <c r="H2" s="27"/>
     </row>
     <row r="3" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H3" s="27"/>
+      <c r="H3" s="28"/>
     </row>
     <row r="4" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H4" s="27"/>
+      <c r="H4" s="28"/>
     </row>
     <row r="5" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H5" s="27"/>
+      <c r="H5" s="28"/>
     </row>
     <row r="6" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H6" s="27"/>
+      <c r="H6" s="28"/>
     </row>
     <row r="7" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H7" s="27"/>
+      <c r="H7" s="28"/>
     </row>
     <row r="8" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H8" s="27"/>
+      <c r="H8" s="28"/>
     </row>
     <row r="9" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H9" s="27"/>
+      <c r="H9" s="28"/>
     </row>
     <row r="10" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H10" s="26"/>
+      <c r="H10" s="27"/>
     </row>
     <row r="11" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H11" s="27"/>
+      <c r="H11" s="28"/>
     </row>
     <row r="12" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H12" s="27"/>
+      <c r="H12" s="28"/>
     </row>
     <row r="13" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H13" s="27"/>
+      <c r="H13" s="28"/>
     </row>
     <row r="14" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H14" s="26"/>
+      <c r="H14" s="27"/>
     </row>
     <row r="15" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H15" s="26"/>
+      <c r="H15" s="27"/>
     </row>
     <row r="16" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H16" s="26"/>
+      <c r="H16" s="27"/>
     </row>
     <row r="17" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H17" s="26"/>
+      <c r="H17" s="27"/>
     </row>
     <row r="18" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H18" s="26"/>
+      <c r="H18" s="27"/>
     </row>
     <row r="19" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H19" s="26"/>
+      <c r="H19" s="27"/>
     </row>
     <row r="20" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H20" s="26"/>
+      <c r="H20" s="27"/>
     </row>
     <row r="21" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H21" s="27"/>
+      <c r="H21" s="28"/>
     </row>
     <row r="22" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H22" s="27"/>
+      <c r="H22" s="28"/>
     </row>
     <row r="23" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H23" s="27"/>
+      <c r="H23" s="28"/>
     </row>
     <row r="24" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H24" s="27"/>
+      <c r="H24" s="28"/>
     </row>
     <row r="25" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H25" s="26"/>
+      <c r="H25" s="27"/>
     </row>
     <row r="26" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H26" s="26"/>
+      <c r="H26" s="27"/>
     </row>
     <row r="27" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H27" s="27"/>
+      <c r="H27" s="28"/>
     </row>
     <row r="28" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H28" s="27"/>
+      <c r="H28" s="28"/>
     </row>
     <row r="29" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H29" s="27"/>
+      <c r="H29" s="28"/>
     </row>
     <row r="30" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H30" s="27"/>
+      <c r="H30" s="28"/>
     </row>
     <row r="31" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H31" s="27"/>
+      <c r="H31" s="28"/>
     </row>
     <row r="32" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H32" s="26"/>
+      <c r="H32" s="27"/>
     </row>
     <row r="33" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H33" s="27"/>
+      <c r="H33" s="28"/>
     </row>
     <row r="34" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H34" s="27"/>
+      <c r="H34" s="28"/>
     </row>
     <row r="35" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H35" s="27"/>
+      <c r="H35" s="28"/>
     </row>
     <row r="36" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H36" s="26"/>
+      <c r="H36" s="27"/>
     </row>
     <row r="37" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H37" s="26"/>
+      <c r="H37" s="27"/>
     </row>
     <row r="38" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H38" s="26"/>
+      <c r="H38" s="27"/>
     </row>
     <row r="39" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H39" s="26"/>
+      <c r="H39" s="27"/>
     </row>
     <row r="40" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H40" s="26"/>
+      <c r="H40" s="27"/>
     </row>
     <row r="41" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H41" s="26"/>
+      <c r="H41" s="27"/>
     </row>
     <row r="42" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H42" s="27"/>
+      <c r="H42" s="28"/>
     </row>
     <row r="43" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H43" s="27"/>
+      <c r="H43" s="28"/>
     </row>
     <row r="44" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H44" s="27"/>
+      <c r="H44" s="28"/>
     </row>
     <row r="45" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H45" s="27"/>
+      <c r="H45" s="28"/>
     </row>
     <row r="46" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H46" s="27"/>
+      <c r="H46" s="28"/>
     </row>
     <row r="47" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H47" s="27"/>
+      <c r="H47" s="28"/>
     </row>
     <row r="48" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H48" s="27"/>
+      <c r="H48" s="28"/>
     </row>
     <row r="49" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H49" s="27"/>
+      <c r="H49" s="28"/>
     </row>
     <row r="50" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="51" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1532,342 +1535,342 @@
     <row r="65" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="66" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="67" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H67" s="27"/>
+      <c r="H67" s="28"/>
     </row>
     <row r="68" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H68" s="27"/>
+      <c r="H68" s="28"/>
     </row>
     <row r="69" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H69" s="27"/>
+      <c r="H69" s="28"/>
     </row>
     <row r="70" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H70" s="27"/>
+      <c r="H70" s="28"/>
     </row>
     <row r="71" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H71" s="26"/>
+      <c r="H71" s="27"/>
     </row>
     <row r="72" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H72" s="27"/>
+      <c r="H72" s="28"/>
     </row>
     <row r="73" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="74" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H74" s="27"/>
+      <c r="H74" s="28"/>
     </row>
     <row r="75" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H75" s="27"/>
+      <c r="H75" s="28"/>
     </row>
     <row r="76" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H76" s="26"/>
+      <c r="H76" s="27"/>
     </row>
     <row r="77" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H77" s="26"/>
+      <c r="H77" s="27"/>
     </row>
     <row r="78" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H78" s="26"/>
+      <c r="H78" s="27"/>
     </row>
     <row r="79" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H79" s="27"/>
+      <c r="H79" s="28"/>
     </row>
     <row r="80" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H80" s="26"/>
+      <c r="H80" s="27"/>
     </row>
     <row r="81" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H81" s="26"/>
+      <c r="H81" s="27"/>
     </row>
     <row r="82" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H82" s="26"/>
+      <c r="H82" s="27"/>
     </row>
     <row r="83" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H83" s="26"/>
+      <c r="H83" s="27"/>
     </row>
     <row r="84" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H84" s="26"/>
+      <c r="H84" s="27"/>
     </row>
     <row r="85" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H85" s="26"/>
+      <c r="H85" s="27"/>
     </row>
     <row r="86" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H86" s="27"/>
+      <c r="H86" s="28"/>
     </row>
     <row r="87" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H87" s="26"/>
+      <c r="H87" s="27"/>
     </row>
     <row r="88" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H88" s="26"/>
+      <c r="H88" s="27"/>
     </row>
     <row r="89" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H89" s="27"/>
+      <c r="H89" s="28"/>
     </row>
     <row r="90" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H90" s="26"/>
+      <c r="H90" s="27"/>
     </row>
     <row r="91" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H91" s="27"/>
+      <c r="H91" s="28"/>
     </row>
     <row r="92" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H92" s="26"/>
+      <c r="H92" s="27"/>
     </row>
     <row r="93" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H93" s="27"/>
+      <c r="H93" s="28"/>
     </row>
     <row r="94" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H94" s="26"/>
+      <c r="H94" s="27"/>
     </row>
     <row r="95" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H95" s="26"/>
+      <c r="H95" s="27"/>
     </row>
     <row r="96" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H96" s="27"/>
+      <c r="H96" s="28"/>
     </row>
     <row r="97" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H97" s="27"/>
+      <c r="H97" s="28"/>
     </row>
     <row r="98" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H98" s="26"/>
+      <c r="H98" s="27"/>
     </row>
     <row r="99" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H99" s="27"/>
+      <c r="H99" s="28"/>
     </row>
     <row r="100" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H100" s="26"/>
+      <c r="H100" s="27"/>
     </row>
     <row r="101" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H101" s="27"/>
+      <c r="H101" s="28"/>
     </row>
     <row r="102" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H102" s="27"/>
+      <c r="H102" s="28"/>
     </row>
     <row r="103" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H103" s="27"/>
+      <c r="H103" s="28"/>
     </row>
     <row r="104" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H104" s="27"/>
+      <c r="H104" s="28"/>
     </row>
     <row r="105" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H105" s="26"/>
+      <c r="H105" s="27"/>
     </row>
     <row r="106" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H106" s="26"/>
+      <c r="H106" s="27"/>
     </row>
     <row r="107" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H107" s="26"/>
+      <c r="H107" s="27"/>
     </row>
     <row r="108" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H108" s="27"/>
+      <c r="H108" s="28"/>
     </row>
     <row r="109" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H109" s="27"/>
+      <c r="H109" s="28"/>
     </row>
     <row r="110" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H110" s="26"/>
+      <c r="H110" s="27"/>
     </row>
     <row r="111" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H111" s="26"/>
+      <c r="H111" s="27"/>
     </row>
     <row r="112" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H112" s="27"/>
+      <c r="H112" s="28"/>
     </row>
     <row r="113" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H113" s="26"/>
+      <c r="H113" s="27"/>
     </row>
     <row r="114" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H114" s="27"/>
+      <c r="H114" s="28"/>
     </row>
     <row r="115" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H115" s="26"/>
+      <c r="H115" s="27"/>
     </row>
     <row r="116" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H116" s="27"/>
+      <c r="H116" s="28"/>
     </row>
     <row r="117" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H117" s="27"/>
+      <c r="H117" s="28"/>
     </row>
     <row r="118" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H118" s="26"/>
+      <c r="H118" s="27"/>
     </row>
     <row r="119" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H119" s="27"/>
+      <c r="H119" s="28"/>
     </row>
     <row r="120" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H120" s="27"/>
+      <c r="H120" s="28"/>
     </row>
     <row r="121" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H121" s="27"/>
+      <c r="H121" s="28"/>
     </row>
     <row r="122" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H122" s="27"/>
+      <c r="H122" s="28"/>
     </row>
     <row r="123" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H123" s="26"/>
+      <c r="H123" s="27"/>
     </row>
     <row r="124" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H124" s="27"/>
+      <c r="H124" s="28"/>
     </row>
     <row r="125" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H125" s="27"/>
+      <c r="H125" s="28"/>
     </row>
     <row r="126" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H126" s="27"/>
+      <c r="H126" s="28"/>
     </row>
     <row r="127" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H127" s="27"/>
+      <c r="H127" s="28"/>
     </row>
     <row r="128" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H128" s="26"/>
+      <c r="H128" s="27"/>
     </row>
     <row r="129" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H129" s="26"/>
+      <c r="H129" s="27"/>
     </row>
     <row r="130" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H130" s="26"/>
+      <c r="H130" s="27"/>
     </row>
     <row r="131" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H131" s="27"/>
+      <c r="H131" s="28"/>
     </row>
     <row r="132" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H132" s="26"/>
+      <c r="H132" s="27"/>
     </row>
     <row r="133" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H133" s="26"/>
+      <c r="H133" s="27"/>
     </row>
     <row r="134" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H134" s="27"/>
+      <c r="H134" s="28"/>
     </row>
     <row r="135" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H135" s="27"/>
+      <c r="H135" s="28"/>
     </row>
     <row r="136" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H136" s="26"/>
+      <c r="H136" s="27"/>
     </row>
     <row r="137" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H137" s="27"/>
+      <c r="H137" s="28"/>
     </row>
     <row r="138" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H138" s="27"/>
+      <c r="H138" s="28"/>
     </row>
     <row r="139" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H139" s="26"/>
+      <c r="H139" s="27"/>
     </row>
     <row r="140" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H140" s="26"/>
+      <c r="H140" s="27"/>
     </row>
     <row r="141" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="142" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H142" s="27"/>
+      <c r="H142" s="28"/>
     </row>
     <row r="143" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H143" s="27"/>
+      <c r="H143" s="28"/>
     </row>
     <row r="144" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H144" s="26"/>
+      <c r="H144" s="27"/>
     </row>
     <row r="145" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H145" s="27"/>
+      <c r="H145" s="28"/>
     </row>
     <row r="146" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H146" s="27"/>
+      <c r="H146" s="28"/>
     </row>
     <row r="147" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H147" s="26"/>
+      <c r="H147" s="27"/>
     </row>
     <row r="148" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H148" s="27"/>
+      <c r="H148" s="28"/>
     </row>
     <row r="149" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H149" s="26"/>
+      <c r="H149" s="27"/>
     </row>
     <row r="150" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H150" s="26"/>
+      <c r="H150" s="27"/>
     </row>
     <row r="151" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H151" s="27"/>
+      <c r="H151" s="28"/>
     </row>
     <row r="152" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H152" s="27"/>
+      <c r="H152" s="28"/>
     </row>
     <row r="153" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H153" s="27"/>
+      <c r="H153" s="28"/>
     </row>
     <row r="154" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H154" s="27"/>
+      <c r="H154" s="28"/>
     </row>
     <row r="155" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H155" s="27"/>
+      <c r="H155" s="28"/>
     </row>
     <row r="156" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H156" s="26"/>
+      <c r="H156" s="27"/>
     </row>
     <row r="157" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H157" s="26"/>
+      <c r="H157" s="27"/>
     </row>
     <row r="158" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H158" s="27"/>
+      <c r="H158" s="28"/>
     </row>
     <row r="159" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H159" s="26"/>
+      <c r="H159" s="27"/>
     </row>
     <row r="160" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H160" s="27"/>
+      <c r="H160" s="28"/>
     </row>
     <row r="161" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H161" s="26"/>
+      <c r="H161" s="27"/>
     </row>
     <row r="162" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H162" s="26"/>
+      <c r="H162" s="27"/>
     </row>
     <row r="163" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H163" s="27"/>
+      <c r="H163" s="28"/>
     </row>
     <row r="164" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H164" s="27"/>
+      <c r="H164" s="28"/>
     </row>
     <row r="165" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H165" s="26"/>
+      <c r="H165" s="27"/>
     </row>
     <row r="166" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H166" s="26"/>
+      <c r="H166" s="27"/>
     </row>
     <row r="167" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H167" s="26"/>
+      <c r="H167" s="27"/>
     </row>
     <row r="168" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H168" s="27"/>
+      <c r="H168" s="28"/>
     </row>
     <row r="169" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H169" s="27"/>
+      <c r="H169" s="28"/>
     </row>
     <row r="170" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H170" s="26"/>
+      <c r="H170" s="27"/>
     </row>
     <row r="171" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H171" s="27"/>
+      <c r="H171" s="28"/>
     </row>
     <row r="172" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H172" s="27"/>
+      <c r="H172" s="28"/>
     </row>
     <row r="173" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H173" s="26"/>
+      <c r="H173" s="27"/>
     </row>
     <row r="174" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H174" s="26"/>
+      <c r="H174" s="27"/>
     </row>
     <row r="175" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H175" s="26"/>
+      <c r="H175" s="27"/>
     </row>
     <row r="176" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H176" s="28"/>
+      <c r="H176" s="29"/>
     </row>
     <row r="177" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H177" s="27"/>
+      <c r="H177" s="28"/>
     </row>
     <row r="178" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H178" s="26"/>
+      <c r="H178" s="27"/>
     </row>
     <row r="179" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H179" s="26"/>
+      <c r="H179" s="27"/>
     </row>
     <row r="180" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="H180" s="27"/>
+      <c r="H180" s="28"/>
     </row>
     <row r="181" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="182" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -2501,7 +2504,7 @@
     <row r="810" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="811" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
-  <autoFilter ref="A1:M180"/>
+  <autoFilter ref="A1:N1"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>

<commit_message>
Checkpoint - 27 abril - falta marca de agua en PDF y reogranizar la Generacion de Horas Extra
</commit_message>
<xml_diff>
--- a/models/hora_extra_template.xlsx
+++ b/models/hora_extra_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Revisar_primero" sheetId="1" state="visible" r:id="rId3"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="77">
   <si>
     <t xml:space="preserve">Aplica</t>
   </si>
@@ -164,19 +164,22 @@
     <t xml:space="preserve"> se_labora</t>
   </si>
   <si>
+    <t xml:space="preserve">“Dia Festivo: Decreto”</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> lunch</t>
+  </si>
+  <si>
     <t xml:space="preserve">Zamora Z1 (Cuadrilla. Nro. 6)</t>
   </si>
   <si>
     <t xml:space="preserve">“Dia Festivo: Cantonizacion”</t>
   </si>
   <si>
-    <t xml:space="preserve"> lunch</t>
+    <t xml:space="preserve"> ?</t>
   </si>
   <si>
     <t xml:space="preserve">Zamora Z1 (Cuadrilla. AP Nro. 4)</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> ?</t>
   </si>
   <si>
     <t xml:space="preserve">Zamora (Agencia)</t>
@@ -1068,31 +1071,31 @@
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>46142</v>
+      </c>
+      <c r="C15" s="1" t="s">
         <v>46</v>
-      </c>
-      <c r="B15" s="2" t="n">
-        <v>46300</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>47</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>46121</v>
       </c>
       <c r="E15" s="2"/>
       <c r="J15" s="3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="8" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B16" s="2" t="n">
         <v>46300</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>46122</v>
@@ -1110,9 +1113,11 @@
         <v>46300</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D17" s="2"/>
+        <v>49</v>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>46139</v>
+      </c>
       <c r="E17" s="2"/>
     </row>
     <row r="18" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1123,9 +1128,11 @@
         <v>46300</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D18" s="2"/>
+        <v>49</v>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>46140</v>
+      </c>
       <c r="E18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1133,12 +1140,14 @@
         <v>53</v>
       </c>
       <c r="B19" s="2" t="n">
-        <v>46031</v>
+        <v>46300</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D19" s="2"/>
+        <v>49</v>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>46141</v>
+      </c>
       <c r="E19" s="2"/>
     </row>
     <row r="20" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1146,10 +1155,10 @@
         <v>54</v>
       </c>
       <c r="B20" s="2" t="n">
-        <v>46080</v>
+        <v>46031</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D20" s="2"/>
       <c r="E20" s="2"/>
@@ -1162,7 +1171,7 @@
         <v>46080</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D21" s="2"/>
       <c r="E21" s="2"/>
@@ -1175,7 +1184,7 @@
         <v>46080</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
@@ -1185,10 +1194,10 @@
         <v>57</v>
       </c>
       <c r="B23" s="2" t="n">
-        <v>46319</v>
+        <v>46080</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
@@ -1198,10 +1207,10 @@
         <v>58</v>
       </c>
       <c r="B24" s="2" t="n">
-        <v>46353</v>
+        <v>46319</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
@@ -1211,10 +1220,10 @@
         <v>59</v>
       </c>
       <c r="B25" s="2" t="n">
-        <v>46065</v>
+        <v>46353</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
@@ -1227,7 +1236,7 @@
         <v>46065</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
@@ -1237,10 +1246,10 @@
         <v>61</v>
       </c>
       <c r="B27" s="2" t="n">
-        <v>46251</v>
+        <v>46065</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D27" s="2"/>
       <c r="E27" s="2"/>
@@ -1253,12 +1262,21 @@
         <v>46251</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D28" s="2"/>
       <c r="E28" s="2"/>
     </row>
     <row r="29" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>46251</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>49</v>
+      </c>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
     </row>
@@ -1331,46 +1349,46 @@
   <sheetData>
     <row r="1" s="23" customFormat="true" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="23" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B1" s="23" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C1" s="23" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D1" s="24" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="25" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F1" s="25" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="G1" s="26" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H1" s="23" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="I1" s="23" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="J1" s="23" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="K1" s="23" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="L1" s="23" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="M1" s="23" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="N1" s="23" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="19.15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Hasta fin de mayo, falta migracion a Cloudfare
</commit_message>
<xml_diff>
--- a/models/hora_extra_template.xlsx
+++ b/models/hora_extra_template.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Revisar_primero" sheetId="1" state="visible" r:id="rId3"/>
@@ -1160,7 +1160,9 @@
       <c r="C20" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D20" s="2"/>
+      <c r="D20" s="2" t="n">
+        <v>46160</v>
+      </c>
       <c r="E20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1173,7 +1175,9 @@
       <c r="C21" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D21" s="2"/>
+      <c r="D21" s="2" t="n">
+        <v>46161</v>
+      </c>
       <c r="E21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1186,7 +1190,9 @@
       <c r="C22" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D22" s="2"/>
+      <c r="D22" s="2" t="n">
+        <v>46162</v>
+      </c>
       <c r="E22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1199,7 +1205,9 @@
       <c r="C23" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D23" s="2"/>
+      <c r="D23" s="2" t="n">
+        <v>46163</v>
+      </c>
       <c r="E23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
no es necesario Ioskeva Light, con la regular esta bien
</commit_message>
<xml_diff>
--- a/models/hora_extra_template.xlsx
+++ b/models/hora_extra_template.xlsx
@@ -1220,7 +1220,9 @@
       <c r="C24" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D24" s="2"/>
+      <c r="D24" s="2" t="n">
+        <v>46174</v>
+      </c>
       <c r="E24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="12.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>